<commit_message>
data added for district heating
</commit_message>
<xml_diff>
--- a/data/gen_profiles_pu.xlsx
+++ b/data/gen_profiles_pu.xlsx
@@ -44178,7 +44178,7 @@
         <v>46188.66666666666</v>
       </c>
       <c r="B3978" t="n">
-        <v>0.2756950146156809</v>
+        <v>0.2756950146156807</v>
       </c>
       <c r="C3978" t="n">
         <v>5.2</v>
@@ -48930,7 +48930,7 @@
         <v>46206.66666666666</v>
       </c>
       <c r="B4410" t="n">
-        <v>0.1890819873239854</v>
+        <v>0.1890819873239855</v>
       </c>
       <c r="C4410" t="n">
         <v>5.2</v>
@@ -53143,7 +53143,7 @@
         <v>46222.625</v>
       </c>
       <c r="B4793" t="n">
-        <v>0.2763501229027899</v>
+        <v>0.27635012290279</v>
       </c>
       <c r="C4793" t="n">
         <v>5.3</v>
@@ -61822,7 +61822,7 @@
         <v>46255.5</v>
       </c>
       <c r="B5582" t="n">
-        <v>0.2937252461569582</v>
+        <v>0.2937252461569583</v>
       </c>
       <c r="C5582" t="n">
         <v>5.3</v>
@@ -62031,7 +62031,7 @@
         <v>46256.29166666666</v>
       </c>
       <c r="B5601" t="n">
-        <v>0.1799500364697916</v>
+        <v>0.1799500364697917</v>
       </c>
       <c r="C5601" t="n">
         <v>4.5</v>
@@ -72074,7 +72074,7 @@
         <v>46294.33333333334</v>
       </c>
       <c r="B6514" t="n">
-        <v>0.09610281818576348</v>
+        <v>0.09610281818576345</v>
       </c>
       <c r="C6514" t="n">
         <v>3.6</v>
@@ -74736,7 +74736,7 @@
         <v>46304.41666666666</v>
       </c>
       <c r="B6756" t="n">
-        <v>0.1389854267363009</v>
+        <v>0.1389854267363008</v>
       </c>
       <c r="C6756" t="n">
         <v>4</v>

</xml_diff>